<commit_message>
Add occurrence ranking graphs; flag all-zero German regions
- Bar chart of species ranked by NUTS units with damage vs monitored
- Region x species map of years with damage
- Label Polish district codes as NUTS2 in the ranking tables
- Report notes DE9/DE3/DE5/DE6 report only zeros, likely not reported

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTy5LTvQsgDsUNQTkJXWE9
</commit_message>
<xml_diff>
--- a/outputs/tables/species_nuts_occurrence_ranking.xlsx
+++ b/outputs/tables/species_nuts_occurrence_ranking.xlsx
@@ -55394,7 +55394,7 @@
       </c>
       <c r="C988" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D988" t="inlineStr">
@@ -55448,7 +55448,7 @@
       </c>
       <c r="C989" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D989" t="inlineStr">
@@ -55502,7 +55502,7 @@
       </c>
       <c r="C990" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D990" t="inlineStr">
@@ -55556,7 +55556,7 @@
       </c>
       <c r="C991" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D991" t="inlineStr">
@@ -55610,7 +55610,7 @@
       </c>
       <c r="C992" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D992" t="inlineStr">
@@ -55664,7 +55664,7 @@
       </c>
       <c r="C993" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D993" t="inlineStr">
@@ -55718,7 +55718,7 @@
       </c>
       <c r="C994" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D994" t="inlineStr">
@@ -55772,7 +55772,7 @@
       </c>
       <c r="C995" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D995" t="inlineStr">
@@ -55826,7 +55826,7 @@
       </c>
       <c r="C996" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D996" t="inlineStr">
@@ -55880,7 +55880,7 @@
       </c>
       <c r="C997" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D997" t="inlineStr">
@@ -55934,7 +55934,7 @@
       </c>
       <c r="C998" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D998" t="inlineStr">
@@ -55988,7 +55988,7 @@
       </c>
       <c r="C999" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D999" t="inlineStr">
@@ -56042,7 +56042,7 @@
       </c>
       <c r="C1000" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1000" t="inlineStr">
@@ -56096,7 +56096,7 @@
       </c>
       <c r="C1001" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1001" t="inlineStr">
@@ -56150,7 +56150,7 @@
       </c>
       <c r="C1002" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1002" t="inlineStr">
@@ -56204,7 +56204,7 @@
       </c>
       <c r="C1003" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1003" t="inlineStr">
@@ -56258,7 +56258,7 @@
       </c>
       <c r="C1004" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1004" t="inlineStr">
@@ -56312,7 +56312,7 @@
       </c>
       <c r="C1005" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1005" t="inlineStr">
@@ -56366,7 +56366,7 @@
       </c>
       <c r="C1006" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1006" t="inlineStr">
@@ -56420,7 +56420,7 @@
       </c>
       <c r="C1007" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1007" t="inlineStr">
@@ -56474,7 +56474,7 @@
       </c>
       <c r="C1008" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1008" t="inlineStr">
@@ -56528,7 +56528,7 @@
       </c>
       <c r="C1009" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1009" t="inlineStr">
@@ -56582,7 +56582,7 @@
       </c>
       <c r="C1010" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1010" t="inlineStr">
@@ -56636,7 +56636,7 @@
       </c>
       <c r="C1011" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1011" t="inlineStr">
@@ -56690,7 +56690,7 @@
       </c>
       <c r="C1012" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1012" t="inlineStr">
@@ -56744,7 +56744,7 @@
       </c>
       <c r="C1013" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1013" t="inlineStr">
@@ -56798,7 +56798,7 @@
       </c>
       <c r="C1014" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1014" t="inlineStr">
@@ -56852,7 +56852,7 @@
       </c>
       <c r="C1015" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1015" t="inlineStr">
@@ -56906,7 +56906,7 @@
       </c>
       <c r="C1016" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1016" t="inlineStr">
@@ -56960,7 +56960,7 @@
       </c>
       <c r="C1017" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1017" t="inlineStr">
@@ -57014,7 +57014,7 @@
       </c>
       <c r="C1018" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1018" t="inlineStr">
@@ -57068,7 +57068,7 @@
       </c>
       <c r="C1019" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1019" t="inlineStr">
@@ -57122,7 +57122,7 @@
       </c>
       <c r="C1020" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1020" t="inlineStr">
@@ -57176,7 +57176,7 @@
       </c>
       <c r="C1021" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1021" t="inlineStr">
@@ -57227,7 +57227,7 @@
       </c>
       <c r="C1022" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1022" t="inlineStr">
@@ -57281,7 +57281,7 @@
       </c>
       <c r="C1023" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1023" t="inlineStr">
@@ -57335,7 +57335,7 @@
       </c>
       <c r="C1024" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1024" t="inlineStr">
@@ -57389,7 +57389,7 @@
       </c>
       <c r="C1025" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1025" t="inlineStr">
@@ -57443,7 +57443,7 @@
       </c>
       <c r="C1026" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1026" t="inlineStr">
@@ -57497,7 +57497,7 @@
       </c>
       <c r="C1027" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1027" t="inlineStr">
@@ -57551,7 +57551,7 @@
       </c>
       <c r="C1028" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1028" t="inlineStr">
@@ -57605,7 +57605,7 @@
       </c>
       <c r="C1029" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1029" t="inlineStr">
@@ -57659,7 +57659,7 @@
       </c>
       <c r="C1030" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1030" t="inlineStr">
@@ -57710,7 +57710,7 @@
       </c>
       <c r="C1031" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1031" t="inlineStr">
@@ -57761,7 +57761,7 @@
       </c>
       <c r="C1032" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1032" t="inlineStr">
@@ -57812,7 +57812,7 @@
       </c>
       <c r="C1033" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1033" t="inlineStr">
@@ -57863,7 +57863,7 @@
       </c>
       <c r="C1034" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1034" t="inlineStr">
@@ -57914,7 +57914,7 @@
       </c>
       <c r="C1035" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1035" t="inlineStr">
@@ -57968,7 +57968,7 @@
       </c>
       <c r="C1036" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1036" t="inlineStr">
@@ -58022,7 +58022,7 @@
       </c>
       <c r="C1037" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1037" t="inlineStr">
@@ -58076,7 +58076,7 @@
       </c>
       <c r="C1038" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1038" t="inlineStr">
@@ -58130,7 +58130,7 @@
       </c>
       <c r="C1039" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1039" t="inlineStr">
@@ -58184,7 +58184,7 @@
       </c>
       <c r="C1040" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1040" t="inlineStr">
@@ -58238,7 +58238,7 @@
       </c>
       <c r="C1041" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1041" t="inlineStr">
@@ -58292,7 +58292,7 @@
       </c>
       <c r="C1042" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1042" t="inlineStr">
@@ -58346,7 +58346,7 @@
       </c>
       <c r="C1043" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1043" t="inlineStr">
@@ -58400,7 +58400,7 @@
       </c>
       <c r="C1044" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1044" t="inlineStr">
@@ -58454,7 +58454,7 @@
       </c>
       <c r="C1045" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1045" t="inlineStr">
@@ -58505,7 +58505,7 @@
       </c>
       <c r="C1046" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1046" t="inlineStr">
@@ -58556,7 +58556,7 @@
       </c>
       <c r="C1047" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1047" t="inlineStr">
@@ -58607,7 +58607,7 @@
       </c>
       <c r="C1048" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1048" t="inlineStr">
@@ -58661,7 +58661,7 @@
       </c>
       <c r="C1049" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1049" t="inlineStr">
@@ -58715,7 +58715,7 @@
       </c>
       <c r="C1050" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1050" t="inlineStr">
@@ -58769,7 +58769,7 @@
       </c>
       <c r="C1051" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1051" t="inlineStr">
@@ -58823,7 +58823,7 @@
       </c>
       <c r="C1052" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1052" t="inlineStr">
@@ -58877,7 +58877,7 @@
       </c>
       <c r="C1053" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1053" t="inlineStr">
@@ -58931,7 +58931,7 @@
       </c>
       <c r="C1054" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1054" t="inlineStr">
@@ -58985,7 +58985,7 @@
       </c>
       <c r="C1055" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1055" t="inlineStr">
@@ -59039,7 +59039,7 @@
       </c>
       <c r="C1056" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1056" t="inlineStr">
@@ -59093,7 +59093,7 @@
       </c>
       <c r="C1057" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1057" t="inlineStr">
@@ -59147,7 +59147,7 @@
       </c>
       <c r="C1058" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1058" t="inlineStr">
@@ -59201,7 +59201,7 @@
       </c>
       <c r="C1059" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1059" t="inlineStr">
@@ -59255,7 +59255,7 @@
       </c>
       <c r="C1060" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1060" t="inlineStr">
@@ -59309,7 +59309,7 @@
       </c>
       <c r="C1061" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1061" t="inlineStr">
@@ -59363,7 +59363,7 @@
       </c>
       <c r="C1062" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1062" t="inlineStr">
@@ -59417,7 +59417,7 @@
       </c>
       <c r="C1063" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1063" t="inlineStr">
@@ -59471,7 +59471,7 @@
       </c>
       <c r="C1064" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1064" t="inlineStr">
@@ -59525,7 +59525,7 @@
       </c>
       <c r="C1065" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1065" t="inlineStr">
@@ -59576,7 +59576,7 @@
       </c>
       <c r="C1066" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1066" t="inlineStr">
@@ -59630,7 +59630,7 @@
       </c>
       <c r="C1067" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1067" t="inlineStr">
@@ -59684,7 +59684,7 @@
       </c>
       <c r="C1068" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1068" t="inlineStr">
@@ -59738,7 +59738,7 @@
       </c>
       <c r="C1069" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1069" t="inlineStr">
@@ -59792,7 +59792,7 @@
       </c>
       <c r="C1070" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1070" t="inlineStr">
@@ -59846,7 +59846,7 @@
       </c>
       <c r="C1071" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1071" t="inlineStr">
@@ -59900,7 +59900,7 @@
       </c>
       <c r="C1072" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1072" t="inlineStr">
@@ -59954,7 +59954,7 @@
       </c>
       <c r="C1073" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1073" t="inlineStr">
@@ -60008,7 +60008,7 @@
       </c>
       <c r="C1074" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1074" t="inlineStr">
@@ -60062,7 +60062,7 @@
       </c>
       <c r="C1075" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1075" t="inlineStr">
@@ -60116,7 +60116,7 @@
       </c>
       <c r="C1076" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1076" t="inlineStr">
@@ -60170,7 +60170,7 @@
       </c>
       <c r="C1077" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1077" t="inlineStr">
@@ -60224,7 +60224,7 @@
       </c>
       <c r="C1078" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1078" t="inlineStr">
@@ -60278,7 +60278,7 @@
       </c>
       <c r="C1079" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1079" t="inlineStr">
@@ -60332,7 +60332,7 @@
       </c>
       <c r="C1080" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1080" t="inlineStr">
@@ -60386,7 +60386,7 @@
       </c>
       <c r="C1081" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1081" t="inlineStr">
@@ -60440,7 +60440,7 @@
       </c>
       <c r="C1082" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1082" t="inlineStr">
@@ -60494,7 +60494,7 @@
       </c>
       <c r="C1083" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1083" t="inlineStr">
@@ -60548,7 +60548,7 @@
       </c>
       <c r="C1084" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1084" t="inlineStr">
@@ -60602,7 +60602,7 @@
       </c>
       <c r="C1085" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1085" t="inlineStr">
@@ -60656,7 +60656,7 @@
       </c>
       <c r="C1086" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1086" t="inlineStr">
@@ -60710,7 +60710,7 @@
       </c>
       <c r="C1087" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1087" t="inlineStr">
@@ -60764,7 +60764,7 @@
       </c>
       <c r="C1088" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1088" t="inlineStr">
@@ -60818,7 +60818,7 @@
       </c>
       <c r="C1089" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1089" t="inlineStr">
@@ -60872,7 +60872,7 @@
       </c>
       <c r="C1090" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1090" t="inlineStr">
@@ -60926,7 +60926,7 @@
       </c>
       <c r="C1091" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1091" t="inlineStr">
@@ -60980,7 +60980,7 @@
       </c>
       <c r="C1092" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1092" t="inlineStr">
@@ -61034,7 +61034,7 @@
       </c>
       <c r="C1093" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1093" t="inlineStr">
@@ -61088,7 +61088,7 @@
       </c>
       <c r="C1094" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1094" t="inlineStr">
@@ -61142,7 +61142,7 @@
       </c>
       <c r="C1095" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1095" t="inlineStr">
@@ -61196,7 +61196,7 @@
       </c>
       <c r="C1096" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1096" t="inlineStr">
@@ -61250,7 +61250,7 @@
       </c>
       <c r="C1097" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1097" t="inlineStr">
@@ -61304,7 +61304,7 @@
       </c>
       <c r="C1098" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1098" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C1099" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1099" t="inlineStr">
@@ -61412,7 +61412,7 @@
       </c>
       <c r="C1100" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1100" t="inlineStr">
@@ -61466,7 +61466,7 @@
       </c>
       <c r="C1101" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1101" t="inlineStr">
@@ -61520,7 +61520,7 @@
       </c>
       <c r="C1102" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1102" t="inlineStr">
@@ -61574,7 +61574,7 @@
       </c>
       <c r="C1103" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1103" t="inlineStr">
@@ -61628,7 +61628,7 @@
       </c>
       <c r="C1104" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1104" t="inlineStr">
@@ -61679,7 +61679,7 @@
       </c>
       <c r="C1105" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1105" t="inlineStr">
@@ -61733,7 +61733,7 @@
       </c>
       <c r="C1106" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1106" t="inlineStr">
@@ -61787,7 +61787,7 @@
       </c>
       <c r="C1107" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1107" t="inlineStr">
@@ -61841,7 +61841,7 @@
       </c>
       <c r="C1108" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1108" t="inlineStr">
@@ -61895,7 +61895,7 @@
       </c>
       <c r="C1109" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1109" t="inlineStr">
@@ -61949,7 +61949,7 @@
       </c>
       <c r="C1110" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1110" t="inlineStr">
@@ -62003,7 +62003,7 @@
       </c>
       <c r="C1111" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1111" t="inlineStr">
@@ -62057,7 +62057,7 @@
       </c>
       <c r="C1112" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1112" t="inlineStr">
@@ -62111,7 +62111,7 @@
       </c>
       <c r="C1113" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1113" t="inlineStr">
@@ -62165,7 +62165,7 @@
       </c>
       <c r="C1114" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1114" t="inlineStr">
@@ -62219,7 +62219,7 @@
       </c>
       <c r="C1115" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1115" t="inlineStr">
@@ -62273,7 +62273,7 @@
       </c>
       <c r="C1116" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1116" t="inlineStr">
@@ -62327,7 +62327,7 @@
       </c>
       <c r="C1117" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1117" t="inlineStr">
@@ -62381,7 +62381,7 @@
       </c>
       <c r="C1118" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1118" t="inlineStr">
@@ -62435,7 +62435,7 @@
       </c>
       <c r="C1119" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1119" t="inlineStr">
@@ -62489,7 +62489,7 @@
       </c>
       <c r="C1120" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1120" t="inlineStr">
@@ -62543,7 +62543,7 @@
       </c>
       <c r="C1121" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1121" t="inlineStr">
@@ -62597,7 +62597,7 @@
       </c>
       <c r="C1122" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1122" t="inlineStr">
@@ -62651,7 +62651,7 @@
       </c>
       <c r="C1123" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1123" t="inlineStr">
@@ -62705,7 +62705,7 @@
       </c>
       <c r="C1124" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1124" t="inlineStr">
@@ -62759,7 +62759,7 @@
       </c>
       <c r="C1125" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1125" t="inlineStr">
@@ -62810,7 +62810,7 @@
       </c>
       <c r="C1126" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1126" t="inlineStr">
@@ -62864,7 +62864,7 @@
       </c>
       <c r="C1127" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1127" t="inlineStr">
@@ -62918,7 +62918,7 @@
       </c>
       <c r="C1128" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1128" t="inlineStr">
@@ -62972,7 +62972,7 @@
       </c>
       <c r="C1129" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1129" t="inlineStr">
@@ -63026,7 +63026,7 @@
       </c>
       <c r="C1130" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1130" t="inlineStr">
@@ -63080,7 +63080,7 @@
       </c>
       <c r="C1131" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1131" t="inlineStr">
@@ -63134,7 +63134,7 @@
       </c>
       <c r="C1132" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1132" t="inlineStr">
@@ -63188,7 +63188,7 @@
       </c>
       <c r="C1133" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1133" t="inlineStr">
@@ -63242,7 +63242,7 @@
       </c>
       <c r="C1134" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1134" t="inlineStr">
@@ -63296,7 +63296,7 @@
       </c>
       <c r="C1135" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1135" t="inlineStr">
@@ -63350,7 +63350,7 @@
       </c>
       <c r="C1136" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1136" t="inlineStr">
@@ -63404,7 +63404,7 @@
       </c>
       <c r="C1137" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1137" t="inlineStr">
@@ -63458,7 +63458,7 @@
       </c>
       <c r="C1138" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1138" t="inlineStr">
@@ -63512,7 +63512,7 @@
       </c>
       <c r="C1139" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1139" t="inlineStr">
@@ -63566,7 +63566,7 @@
       </c>
       <c r="C1140" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1140" t="inlineStr">
@@ -63620,7 +63620,7 @@
       </c>
       <c r="C1141" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1141" t="inlineStr">
@@ -63674,7 +63674,7 @@
       </c>
       <c r="C1142" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1142" t="inlineStr">
@@ -63728,7 +63728,7 @@
       </c>
       <c r="C1143" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1143" t="inlineStr">
@@ -63782,7 +63782,7 @@
       </c>
       <c r="C1144" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1144" t="inlineStr">
@@ -63836,7 +63836,7 @@
       </c>
       <c r="C1145" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1145" t="inlineStr">
@@ -63890,7 +63890,7 @@
       </c>
       <c r="C1146" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1146" t="inlineStr">
@@ -63944,7 +63944,7 @@
       </c>
       <c r="C1147" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1147" t="inlineStr">
@@ -63998,7 +63998,7 @@
       </c>
       <c r="C1148" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1148" t="inlineStr">
@@ -64052,7 +64052,7 @@
       </c>
       <c r="C1149" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1149" t="inlineStr">
@@ -64106,7 +64106,7 @@
       </c>
       <c r="C1150" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1150" t="inlineStr">
@@ -64160,7 +64160,7 @@
       </c>
       <c r="C1151" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1151" t="inlineStr">
@@ -64214,7 +64214,7 @@
       </c>
       <c r="C1152" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1152" t="inlineStr">
@@ -64268,7 +64268,7 @@
       </c>
       <c r="C1153" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1153" t="inlineStr">
@@ -64322,7 +64322,7 @@
       </c>
       <c r="C1154" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1154" t="inlineStr">
@@ -64376,7 +64376,7 @@
       </c>
       <c r="C1155" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1155" t="inlineStr">
@@ -64430,7 +64430,7 @@
       </c>
       <c r="C1156" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1156" t="inlineStr">
@@ -64481,7 +64481,7 @@
       </c>
       <c r="C1157" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1157" t="inlineStr">
@@ -64535,7 +64535,7 @@
       </c>
       <c r="C1158" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1158" t="inlineStr">
@@ -64589,7 +64589,7 @@
       </c>
       <c r="C1159" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1159" t="inlineStr">
@@ -64643,7 +64643,7 @@
       </c>
       <c r="C1160" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1160" t="inlineStr">
@@ -64697,7 +64697,7 @@
       </c>
       <c r="C1161" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1161" t="inlineStr">
@@ -64751,7 +64751,7 @@
       </c>
       <c r="C1162" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1162" t="inlineStr">
@@ -64805,7 +64805,7 @@
       </c>
       <c r="C1163" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1163" t="inlineStr">
@@ -64859,7 +64859,7 @@
       </c>
       <c r="C1164" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1164" t="inlineStr">
@@ -64913,7 +64913,7 @@
       </c>
       <c r="C1165" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1165" t="inlineStr">
@@ -64967,7 +64967,7 @@
       </c>
       <c r="C1166" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1166" t="inlineStr">
@@ -65021,7 +65021,7 @@
       </c>
       <c r="C1167" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1167" t="inlineStr">
@@ -65075,7 +65075,7 @@
       </c>
       <c r="C1168" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1168" t="inlineStr">
@@ -65129,7 +65129,7 @@
       </c>
       <c r="C1169" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1169" t="inlineStr">
@@ -65183,7 +65183,7 @@
       </c>
       <c r="C1170" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1170" t="inlineStr">
@@ -65237,7 +65237,7 @@
       </c>
       <c r="C1171" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1171" t="inlineStr">
@@ -65291,7 +65291,7 @@
       </c>
       <c r="C1172" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1172" t="inlineStr">
@@ -65345,7 +65345,7 @@
       </c>
       <c r="C1173" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1173" t="inlineStr">
@@ -65399,7 +65399,7 @@
       </c>
       <c r="C1174" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1174" t="inlineStr">
@@ -65453,7 +65453,7 @@
       </c>
       <c r="C1175" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1175" t="inlineStr">
@@ -65507,7 +65507,7 @@
       </c>
       <c r="C1176" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1176" t="inlineStr">
@@ -65561,7 +65561,7 @@
       </c>
       <c r="C1177" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1177" t="inlineStr">
@@ -65615,7 +65615,7 @@
       </c>
       <c r="C1178" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1178" t="inlineStr">
@@ -65669,7 +65669,7 @@
       </c>
       <c r="C1179" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1179" t="inlineStr">
@@ -65723,7 +65723,7 @@
       </c>
       <c r="C1180" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1180" t="inlineStr">
@@ -65777,7 +65777,7 @@
       </c>
       <c r="C1181" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1181" t="inlineStr">
@@ -65831,7 +65831,7 @@
       </c>
       <c r="C1182" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1182" t="inlineStr">
@@ -65885,7 +65885,7 @@
       </c>
       <c r="C1183" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1183" t="inlineStr">
@@ -65939,7 +65939,7 @@
       </c>
       <c r="C1184" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1184" t="inlineStr">
@@ -65993,7 +65993,7 @@
       </c>
       <c r="C1185" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1185" t="inlineStr">
@@ -66047,7 +66047,7 @@
       </c>
       <c r="C1186" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1186" t="inlineStr">
@@ -66101,7 +66101,7 @@
       </c>
       <c r="C1187" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1187" t="inlineStr">
@@ -66155,7 +66155,7 @@
       </c>
       <c r="C1188" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1188" t="inlineStr">
@@ -66209,7 +66209,7 @@
       </c>
       <c r="C1189" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1189" t="inlineStr">
@@ -66263,7 +66263,7 @@
       </c>
       <c r="C1190" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1190" t="inlineStr">
@@ -66317,7 +66317,7 @@
       </c>
       <c r="C1191" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1191" t="inlineStr">
@@ -66371,7 +66371,7 @@
       </c>
       <c r="C1192" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1192" t="inlineStr">
@@ -66425,7 +66425,7 @@
       </c>
       <c r="C1193" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1193" t="inlineStr">
@@ -66479,7 +66479,7 @@
       </c>
       <c r="C1194" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1194" t="inlineStr">
@@ -66533,7 +66533,7 @@
       </c>
       <c r="C1195" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1195" t="inlineStr">
@@ -66587,7 +66587,7 @@
       </c>
       <c r="C1196" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1196" t="inlineStr">
@@ -66641,7 +66641,7 @@
       </c>
       <c r="C1197" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1197" t="inlineStr">
@@ -66695,7 +66695,7 @@
       </c>
       <c r="C1198" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1198" t="inlineStr">
@@ -66749,7 +66749,7 @@
       </c>
       <c r="C1199" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1199" t="inlineStr">
@@ -66803,7 +66803,7 @@
       </c>
       <c r="C1200" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1200" t="inlineStr">
@@ -66857,7 +66857,7 @@
       </c>
       <c r="C1201" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1201" t="inlineStr">
@@ -66911,7 +66911,7 @@
       </c>
       <c r="C1202" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1202" t="inlineStr">
@@ -66965,7 +66965,7 @@
       </c>
       <c r="C1203" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1203" t="inlineStr">
@@ -67019,7 +67019,7 @@
       </c>
       <c r="C1204" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1204" t="inlineStr">
@@ -67073,7 +67073,7 @@
       </c>
       <c r="C1205" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1205" t="inlineStr">
@@ -67127,7 +67127,7 @@
       </c>
       <c r="C1206" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1206" t="inlineStr">
@@ -67181,7 +67181,7 @@
       </c>
       <c r="C1207" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1207" t="inlineStr">
@@ -67235,7 +67235,7 @@
       </c>
       <c r="C1208" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D1208" t="inlineStr">
@@ -72423,7 +72423,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D57">
@@ -72479,7 +72479,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D58">
@@ -72535,7 +72535,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D59">
@@ -72591,7 +72591,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D60">
@@ -72647,7 +72647,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D61">
@@ -72703,7 +72703,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D62">
@@ -72759,7 +72759,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D63">
@@ -72815,7 +72815,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D64">
@@ -72871,7 +72871,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D65">
@@ -72927,7 +72927,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D66">
@@ -72983,7 +72983,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D67">
@@ -73039,7 +73039,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D68">
@@ -73095,7 +73095,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D69">
@@ -73151,7 +73151,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D70">
@@ -73207,7 +73207,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D71">
@@ -73263,7 +73263,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D72">
@@ -73319,7 +73319,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>NUTS1</t>
+          <t>NUTS2</t>
         </is>
       </c>
       <c r="D73">

</xml_diff>